<commit_message>
v23 Phase 104: Lead-Management V2 Fundament (PLAN_LEAD_V2)
Datenmodell (Objektart, ad_id, Vorab-Angebot, Terminarten, ICS-UID,
Kompetenzen/Handelsvertreter am AD-Profil, todos, info_veranstaltungen,
benutzer_einstellungen), Sparte GW, Steuerdatei (Kaskade 5 Stufen, Gruende
verloren/Nachbearbeitung, Blaetter Objektarten + Status), Parameter,
Mail-Vorlagen disqualifiziert/online_termin_einladung, lead_info
(Terminregel NRW-Feiertage), lead_v2 (Helfer), Migration v23, Router-Stubs.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/leadmanagement_logik_v1.xlsx
+++ b/leadmanagement_logik_v1.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Kaskade" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Gruende" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Wunschzeiten" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Objektarten" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Status" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -504,7 +506,6 @@
           <t>janein</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>J</t>
@@ -513,7 +514,6 @@
       <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>nein</t>
@@ -559,7 +559,6 @@
           <t>O01</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -582,7 +581,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>N</t>
@@ -596,7 +594,6 @@
           <t>O02</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -619,7 +616,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>N</t>
@@ -633,7 +629,6 @@
           <t>O05</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -674,7 +669,6 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -697,7 +691,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>N</t>
@@ -711,7 +704,6 @@
           <t>A02</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -734,7 +726,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>J</t>
@@ -748,7 +739,6 @@
           <t>A03</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -771,7 +761,6 @@
           <t>janein</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>N</t>
@@ -780,8 +769,6 @@
       <c r="G9" t="n">
         <v>8</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -822,7 +809,6 @@
           <t>H02</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -858,8 +844,6 @@
       <c r="G11" t="n">
         <v>10</v>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -895,8 +879,6 @@
       <c r="G12" t="n">
         <v>11</v>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -919,7 +901,6 @@
           <t>janein</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>N</t>
@@ -928,8 +909,6 @@
       <c r="G13" t="n">
         <v>12</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -965,8 +944,6 @@
       <c r="G14" t="n">
         <v>13</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1002,8 +979,6 @@
       <c r="G15" t="n">
         <v>14</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1026,7 +1001,6 @@
           <t>janein</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>J</t>
@@ -1035,7 +1009,6 @@
       <c r="G16" t="n">
         <v>1</v>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>nein</t>
@@ -1081,7 +1054,6 @@
           <t>PO01</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1122,7 +1094,6 @@
           <t>PD01</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1158,8 +1129,6 @@
       <c r="G19" t="n">
         <v>4</v>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1182,7 +1151,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>N</t>
@@ -1191,8 +1159,6 @@
       <c r="G20" t="n">
         <v>5</v>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1228,8 +1194,6 @@
       <c r="G21" t="n">
         <v>6</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1252,7 +1216,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>J</t>
@@ -1266,7 +1229,6 @@
           <t>PO04</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1302,8 +1264,6 @@
       <c r="G23" t="n">
         <v>8</v>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1339,8 +1299,6 @@
       <c r="G24" t="n">
         <v>9</v>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1376,8 +1334,6 @@
       <c r="G25" t="n">
         <v>10</v>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1400,7 +1356,6 @@
           <t>janein</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>N</t>
@@ -1409,8 +1364,6 @@
       <c r="G26" t="n">
         <v>11</v>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1446,8 +1399,6 @@
       <c r="G27" t="n">
         <v>12</v>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1470,7 +1421,6 @@
           <t>janein</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>J</t>
@@ -1511,7 +1461,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>J</t>
@@ -1525,7 +1474,6 @@
           <t>KO05</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1548,7 +1496,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>N</t>
@@ -1557,8 +1504,6 @@
       <c r="G30" t="n">
         <v>3</v>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1594,8 +1539,6 @@
       <c r="G31" t="n">
         <v>4</v>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1631,8 +1574,6 @@
       <c r="G32" t="n">
         <v>5</v>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1668,8 +1609,6 @@
       <c r="G33" t="n">
         <v>6</v>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1692,7 +1631,6 @@
           <t>janein</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>J</t>
@@ -1701,8 +1639,6 @@
       <c r="G34" t="n">
         <v>1</v>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1738,8 +1674,6 @@
       <c r="G35" t="n">
         <v>2</v>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1762,7 +1696,6 @@
           <t>zahl</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>N</t>
@@ -1771,8 +1704,6 @@
       <c r="G36" t="n">
         <v>3</v>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1808,8 +1739,6 @@
       <c r="G37" t="n">
         <v>4</v>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1845,8 +1774,6 @@
       <c r="G38" t="n">
         <v>5</v>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1882,8 +1809,6 @@
       <c r="G39" t="n">
         <v>6</v>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1966,7 +1891,6 @@
       <c r="C3" t="n">
         <v>20</v>
       </c>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1982,7 +1906,6 @@
       <c r="C4" t="n">
         <v>10</v>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1998,7 +1921,6 @@
       <c r="C5" t="n">
         <v>15</v>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2014,7 +1936,6 @@
       <c r="C6" t="n">
         <v>15</v>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2030,7 +1951,6 @@
       <c r="C7" t="n">
         <v>5</v>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2046,7 +1966,6 @@
       <c r="C8" t="n">
         <v>10</v>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2062,7 +1981,6 @@
       <c r="C9" t="n">
         <v>25</v>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2078,7 +1996,6 @@
       <c r="C10" t="n">
         <v>20</v>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2094,7 +2011,6 @@
       <c r="C11" t="n">
         <v>10</v>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2110,7 +2026,6 @@
       <c r="C12" t="n">
         <v>5</v>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2126,7 +2041,6 @@
       <c r="C13" t="n">
         <v>10</v>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2142,7 +2056,6 @@
       <c r="C14" t="n">
         <v>-10</v>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2158,7 +2071,6 @@
       <c r="C15" t="n">
         <v>5</v>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2194,7 +2106,6 @@
       <c r="C17" t="n">
         <v>15</v>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2210,7 +2121,6 @@
       <c r="C18" t="n">
         <v>10</v>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2226,7 +2136,6 @@
       <c r="C19" t="n">
         <v>10</v>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2242,7 +2151,6 @@
       <c r="C20" t="n">
         <v>10</v>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2258,7 +2166,6 @@
       <c r="C21" t="n">
         <v>10</v>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2274,7 +2181,6 @@
       <c r="C22" t="n">
         <v>25</v>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2290,7 +2196,6 @@
       <c r="C23" t="n">
         <v>20</v>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2306,7 +2211,6 @@
       <c r="C24" t="n">
         <v>10</v>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2322,7 +2226,6 @@
       <c r="C25" t="n">
         <v>25</v>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2338,7 +2241,6 @@
       <c r="C26" t="n">
         <v>20</v>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2354,7 +2256,6 @@
       <c r="C27" t="n">
         <v>10</v>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2370,7 +2271,6 @@
       <c r="C28" t="n">
         <v>25</v>
       </c>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2386,7 +2286,6 @@
       <c r="C29" t="n">
         <v>20</v>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2402,7 +2301,6 @@
       <c r="C30" t="n">
         <v>10</v>
       </c>
-      <c r="D30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2482,7 +2380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2594,6 +2492,26 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>+14d</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>mail_disqualifiziert</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>J</t>
         </is>
       </c>
@@ -2609,7 +2527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2975,6 +2893,108 @@
         </is>
       </c>
       <c r="C21" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>zurueckgestellt</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Nachbearbeitung, noch nicht bereit für VOT</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>verloren</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Zu teuer</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>verloren</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Kein Interesse mehr</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>verloren</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bleibt bei Öl/Gas</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>verloren</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Woanders unterschrieben</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>verloren</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>J</t>
         </is>
@@ -3143,4 +3163,528 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>bezeichnung</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>parteien_pflicht</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>erfassungs_wert</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EFH</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Einfamilienhaus</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Einfamilienhaus</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RH</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Reihenhaus</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Reihenhaus</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Reihenendhaus</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reihenhaus</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MFH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mehrfamilienhaus</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mehrfamilienhaus</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>farbe</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>board</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>gruppe</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>monday_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>#9aa4b2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>hauptboard</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Neuer Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>in_kontaktierung</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>In Kontaktierung</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>#e87ba4</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>hauptboard</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1. Kontaktversuch|2. Kontaktversuch|3. Kontaktversuch|4. Kontaktversuch|5. Kontaktversuch|erneuter Anruf|Telefongespräch|E-Mail|WhatsApp</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>qualifiziert</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Qualifiziert</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>#2a78d6</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>hauptboard</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>zurueckgestellt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Zurückgestellt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>#c9a227</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>hauptboard</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>pausiert</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Standby|Will sich selber zurückmelden|Nachbearbeitung</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>nicht_erreicht</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Nicht erreicht</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>#e05c8a</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>hauptboard</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>disqualifiziert</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Disqualifiziert - nicht erreicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>unqualifiziert</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Unqualifiziert</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#d64545</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>hauptboard</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>disqualifiziert</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Disqualifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>terminiert</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Terminiert</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>#7bc96f</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>terminiert</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>angebotserstellung</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Terminiert|Teams Meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Erfasst</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>#5b6b8a</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>terminiert</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>angebotserstellung</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Angebotserstellung|Vorab Angebot</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>angebot</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Angebot</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>#a0714f</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>terminiert</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>angebotsversand</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Angebot versendet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>gewonnen</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Gewonnen</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>#1baf7a</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>terminiert</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>gewonnen</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>verloren</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Verloren</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>#6b7280</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>terminiert</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>verloren</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>